<commit_message>
Modified quote items template to include space in UnitPrice
</commit_message>
<xml_diff>
--- a/quote_items_template.xlsx
+++ b/quote_items_template.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Staff\Documents\Other\Vutivi\Quote2Cash\Code\Quote2Cash\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Staff\Documents\Other\Vutivi\Biture\Code\biture\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A5AC04D-0627-49C5-B8B3-94BC9C75298F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6253DB74-D44F-4E5F-BC80-EF5D60EF6684}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,10 +36,10 @@
     <t>Description</t>
   </si>
   <si>
-    <t>UnitPrice</t>
-  </si>
-  <si>
     <t>Code</t>
+  </si>
+  <si>
+    <t>Unit Price</t>
   </si>
 </sst>
 </file>
@@ -358,14 +358,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
@@ -374,7 +374,7 @@
         <v>2</v>
       </c>
       <c r="E1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>